<commit_message>
Update WRCF automation, docs, and trackers
</commit_message>
<xml_diff>
--- a/temp/WRCF End-to-End Test Cases_reverified.xlsx
+++ b/temp/WRCF End-to-End Test Cases_reverified.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Execution Legend" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Manage WRCF" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="FG" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="PWO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SWO" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="CI Mapping" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Manage WRCF Skills" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Skills" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Task" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Control Point" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Roles" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Role Mapping" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Companies" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Legend" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manage WRCF" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FG" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PWO" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWO" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI Mapping" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manage WRCF Skills" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skills" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control Point" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Mapping" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Companies" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Roles'!$A$1:$N$1</definedName>
@@ -1176,27 +1176,27 @@
       </c>
       <c r="U1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 03:41 PM @ 02/04/26</t>
+          <t>Test run 03:41 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 03:46 PM @ 02/04/26</t>
+          <t>Test run 03:46 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 04:23 PM @ 02/04/26</t>
+          <t>Test run 04:23 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>Test run @ 08:17 PM @ 02/04/26</t>
+          <t>Test run 08:17 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -3119,22 +3119,22 @@
       </c>
       <c r="U1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 04:23 PM @ 02/04/26</t>
+          <t>Test run 04:23 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Test run @ 07:46 PM @ 02/04/26</t>
+          <t>Test run 07:46 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Test run @ 08:17 PM @ 02/04/26</t>
+          <t>Test run 08:17 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -4915,22 +4915,22 @@
       </c>
       <c r="U1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" s="31" t="inlineStr">
         <is>
-          <t>Test run @ 10:13 PM @ 02/04/26</t>
+          <t>Test run 10:13 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Test run @ 10:46 PM @ 02/04/26</t>
+          <t>Test run 10:46 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Test run @ 11:09 PM @ 02/04/26</t>
+          <t>Test run 11:09 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -6646,22 +6646,22 @@
       </c>
       <c r="U1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>Test run @ 10:25 PM @ 02/04/26</t>
+          <t>Test run 10:25 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Test run @ 10:46 PM @ 02/04/26</t>
+          <t>Test run 10:46 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Test run @ 11:09 PM @ 02/04/26</t>
+          <t>Test run 11:09 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="U1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -10723,22 +10723,22 @@
       </c>
       <c r="U1" s="26" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" s="26" t="inlineStr">
         <is>
-          <t>Test run @ 03:01 PM @ 02/04/26</t>
+          <t>Test run 03:01 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Test run @ 09:40 PM @ 02/04/26</t>
+          <t>Test run 09:40 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Test run @ 09:45 PM @ 02/04/26</t>
+          <t>Test run 09:45 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -14205,22 +14205,22 @@
       </c>
       <c r="U1" s="26" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" s="26" t="inlineStr">
         <is>
-          <t>Test run @ 03:05 PM @ 02/04/26</t>
+          <t>Test run 03:05 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Test run @ 09:40 PM @ 02/04/26</t>
+          <t>Test run 09:40 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Test run @ 09:45 PM @ 02/04/26</t>
+          <t>Test run 09:45 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -18754,27 +18754,27 @@
       </c>
       <c r="U1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 03:24 PM @ 02/04/26</t>
+          <t>Test run 03:24 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 03:38 PM @ 02/04/26</t>
+          <t>Test run 03:38 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 04:23 PM @ 02/04/26</t>
+          <t>Test run 04:23 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>Test run @ 08:17 PM @ 02/04/26</t>
+          <t>Test run 08:17 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -22095,22 +22095,22 @@
       </c>
       <c r="U1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 03:24 PM @ 02/04/26</t>
+          <t>Test run 03:24 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 04:23 PM @ 02/04/26</t>
+          <t>Test run 04:23 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Test run @ 08:17 PM @ 02/04/26</t>
+          <t>Test run 08:17 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -24692,22 +24692,22 @@
       </c>
       <c r="U1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 03:24 PM @ 02/04/26</t>
+          <t>Test run 03:24 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 04:23 PM @ 02/04/26</t>
+          <t>Test run 04:23 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Test run @ 08:17 PM @ 02/04/26</t>
+          <t>Test run 08:17 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -27288,27 +27288,27 @@
       </c>
       <c r="U1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 03:24 PM @ 02/04/26</t>
+          <t>Test run 03:24 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 04:23 PM @ 02/04/26</t>
+          <t>Test run 04:23 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 04:32 PM @ 02/04/26</t>
+          <t>Test run 04:32 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>Test run @ 08:17 PM @ 02/04/26</t>
+          <t>Test run 08:17 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -31899,22 +31899,22 @@
       </c>
       <c r="U1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 03:41 PM @ 02/04/26</t>
+          <t>Test run 03:41 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 04:23 PM @ 02/04/26</t>
+          <t>Test run 04:23 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Test run @ 08:17 PM @ 02/04/26</t>
+          <t>Test run 08:17 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>
@@ -33278,22 +33278,22 @@
       </c>
       <c r="U1" s="25" t="inlineStr">
         <is>
-          <t>Test run @ 11:41 PM @ 01/04/26</t>
+          <t>Test run 11:41 PM 01/04/26 (local)</t>
         </is>
       </c>
       <c r="V1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 03:41 PM @ 02/04/26</t>
+          <t>Test run 03:41 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="W1" s="27" t="inlineStr">
         <is>
-          <t>Test run @ 04:23 PM @ 02/04/26</t>
+          <t>Test run 04:23 PM 02/04/26 (local)</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Test run @ 08:17 PM @ 02/04/26</t>
+          <t>Test run 08:17 PM 02/04/26 (local)</t>
         </is>
       </c>
     </row>

</xml_diff>